<commit_message>
Add auth system, admin panel, quote isolation, logout modal
</commit_message>
<xml_diff>
--- a/Order.xlsx
+++ b/Order.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aghya\Desktop\Athena Marine\Athena\internal-quote-system\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86F83FDB-D60C-4E12-ABA9-E7825BDFDC5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA5871AF-0861-4EAE-ADC7-AF9615CF6178}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,28 +33,6 @@
     </ext>
   </extLst>
 </workbook>
-</file>
-
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
-  <metadataTypes count="1">
-    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <valueMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </valueMetadata>
-</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -464,147 +442,147 @@
     <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -622,70 +600,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
-<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
-  <global>
-    <keyFlags>
-      <key name="_Self">
-        <flag name="ExcludeFromFile" value="1"/>
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_DisplayString">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Flags">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Format">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_SubLabel">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Attribution">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Icon">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Display">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_CanonicalPropertyNames">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_ClassificationId">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-    </keyFlags>
-  </global>
-</rvTypesInfo>
-</file>
-
-<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-  </rv>
-</rvData>
-</file>
-
-<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
-<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
-  <s t="_localImage">
-    <k n="_rvRel:LocalImageIdentifier" t="i"/>
-    <k n="CalcOrigin" t="i"/>
-  </s>
-</rvStructures>
-</file>
-
-<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
-<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <rel r:id="rId1"/>
-</richValueRels>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -985,122 +899,120 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="22"/>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
+      <c r="A1" s="43"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
     </row>
     <row r="2" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="39"/>
-      <c r="B2" s="39"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
+      <c r="A2" s="26"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
     </row>
     <row r="3" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="31" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
-      <c r="B3" s="27"/>
-      <c r="C3" s="56" t="s">
-        <v>0</v>
-      </c>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
+      <c r="A3" s="37"/>
+      <c r="B3" s="38"/>
+      <c r="C3" s="42" t="s">
+        <v>0</v>
+      </c>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="28"/>
     </row>
     <row r="4" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="27"/>
-      <c r="B4" s="27"/>
-      <c r="C4" s="58" t="s">
+      <c r="A4" s="38"/>
+      <c r="B4" s="38"/>
+      <c r="C4" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="57"/>
-      <c r="E4" s="57"/>
-      <c r="F4" s="57"/>
-      <c r="G4" s="57"/>
-      <c r="H4" s="57"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28"/>
+      <c r="G4" s="28"/>
+      <c r="H4" s="28"/>
     </row>
     <row r="5" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="27"/>
-      <c r="B5" s="27"/>
-      <c r="C5" s="59" t="s">
+      <c r="A5" s="38"/>
+      <c r="B5" s="38"/>
+      <c r="C5" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="57"/>
-      <c r="E5" s="57"/>
-      <c r="F5" s="57"/>
-      <c r="G5" s="57"/>
-      <c r="H5" s="57"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="28"/>
+      <c r="G5" s="28"/>
+      <c r="H5" s="28"/>
     </row>
     <row r="6" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="27"/>
-      <c r="B6" s="27"/>
-      <c r="C6" s="60" t="s">
+      <c r="A6" s="38"/>
+      <c r="B6" s="38"/>
+      <c r="C6" s="31" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="57"/>
-      <c r="E6" s="57"/>
-      <c r="F6" s="60"/>
-      <c r="G6" s="57"/>
-      <c r="H6" s="57"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="28"/>
+      <c r="F6" s="31"/>
+      <c r="G6" s="28"/>
+      <c r="H6" s="28"/>
     </row>
     <row r="7" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="27"/>
-      <c r="B7" s="27"/>
-      <c r="C7" s="59" t="s">
+      <c r="A7" s="38"/>
+      <c r="B7" s="38"/>
+      <c r="C7" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="57"/>
-      <c r="E7" s="57"/>
-      <c r="F7" s="60" t="s">
+      <c r="D7" s="28"/>
+      <c r="E7" s="28"/>
+      <c r="F7" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="G7" s="57"/>
-      <c r="H7" s="57"/>
+      <c r="G7" s="28"/>
+      <c r="H7" s="28"/>
     </row>
     <row r="8" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="39"/>
-      <c r="B8" s="39"/>
-      <c r="C8" s="39"/>
-      <c r="D8" s="39"/>
-      <c r="E8" s="39"/>
-      <c r="F8" s="39"/>
-      <c r="G8" s="39"/>
-      <c r="H8" s="39"/>
+      <c r="A8" s="26"/>
+      <c r="B8" s="26"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="26"/>
     </row>
     <row r="9" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="29" t="s">
+      <c r="A9" s="46" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="25"/>
-      <c r="C9" s="25"/>
-      <c r="D9" s="25"/>
-      <c r="E9" s="25"/>
-      <c r="F9" s="25"/>
-      <c r="G9" s="26" t="s">
+      <c r="B9" s="47"/>
+      <c r="C9" s="47"/>
+      <c r="D9" s="47"/>
+      <c r="E9" s="47"/>
+      <c r="F9" s="47"/>
+      <c r="G9" s="45" t="s">
         <v>39</v>
       </c>
-      <c r="H9" s="27"/>
+      <c r="H9" s="38"/>
     </row>
     <row r="10" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="25"/>
-      <c r="B10" s="25"/>
-      <c r="C10" s="25"/>
-      <c r="D10" s="25"/>
-      <c r="E10" s="25"/>
-      <c r="F10" s="25"/>
-      <c r="G10" s="27"/>
-      <c r="H10" s="27"/>
+      <c r="A10" s="47"/>
+      <c r="B10" s="47"/>
+      <c r="C10" s="47"/>
+      <c r="D10" s="47"/>
+      <c r="E10" s="47"/>
+      <c r="F10" s="47"/>
+      <c r="G10" s="38"/>
+      <c r="H10" s="38"/>
     </row>
     <row r="11" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5"/>
@@ -1113,126 +1025,126 @@
       <c r="H11" s="5"/>
     </row>
     <row r="12" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="28" t="s">
+      <c r="A12" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="B12" s="13"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="28" t="s">
+      <c r="B12" s="30"/>
+      <c r="C12" s="30"/>
+      <c r="D12" s="30"/>
+      <c r="E12" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
-      <c r="H12" s="13"/>
+      <c r="F12" s="30"/>
+      <c r="G12" s="30"/>
+      <c r="H12" s="30"/>
     </row>
     <row r="13" spans="1:8" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="51" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="13"/>
-      <c r="C13" s="40" t="str">
+      <c r="B13" s="30"/>
+      <c r="C13" s="29" t="str">
         <f>G9</f>
         <v xml:space="preserve">Quote Ref: </v>
       </c>
-      <c r="D13" s="13"/>
-      <c r="E13" s="10" t="s">
+      <c r="D13" s="30"/>
+      <c r="E13" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="F13" s="11"/>
-      <c r="G13" s="24"/>
-      <c r="H13" s="11"/>
+      <c r="F13" s="33"/>
+      <c r="G13" s="34"/>
+      <c r="H13" s="33"/>
     </row>
     <row r="14" spans="1:8" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="15" t="s">
+      <c r="A14" s="40" t="s">
         <v>5</v>
       </c>
-      <c r="B14" s="13"/>
-      <c r="C14" s="16">
+      <c r="B14" s="30"/>
+      <c r="C14" s="48">
         <f ca="1">TODAY()</f>
-        <v>46181</v>
-      </c>
-      <c r="D14" s="11"/>
-      <c r="E14" s="10" t="s">
+        <v>46183</v>
+      </c>
+      <c r="D14" s="33"/>
+      <c r="E14" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="F14" s="11"/>
-      <c r="G14" s="35"/>
-      <c r="H14" s="11"/>
+      <c r="F14" s="33"/>
+      <c r="G14" s="41"/>
+      <c r="H14" s="33"/>
     </row>
     <row r="15" spans="1:8" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="40" t="s">
         <v>6</v>
       </c>
-      <c r="B15" s="13"/>
-      <c r="C15" s="16">
+      <c r="B15" s="30"/>
+      <c r="C15" s="48">
         <f ca="1">TODAY()+30</f>
-        <v>46211</v>
-      </c>
-      <c r="D15" s="11"/>
-      <c r="E15" s="10" t="s">
+        <v>46213</v>
+      </c>
+      <c r="D15" s="33"/>
+      <c r="E15" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="F15" s="11"/>
-      <c r="G15" s="24"/>
-      <c r="H15" s="11"/>
+      <c r="F15" s="33"/>
+      <c r="G15" s="34"/>
+      <c r="H15" s="33"/>
     </row>
     <row r="16" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
-      <c r="E16" s="10" t="s">
+      <c r="E16" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="F16" s="11"/>
-      <c r="G16" s="16"/>
-      <c r="H16" s="21"/>
+      <c r="F16" s="33"/>
+      <c r="G16" s="48"/>
+      <c r="H16" s="60"/>
     </row>
     <row r="17" spans="1:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5"/>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
       <c r="D17" s="5"/>
-      <c r="E17" s="10" t="s">
+      <c r="E17" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="F17" s="11"/>
-      <c r="G17" s="24"/>
-      <c r="H17" s="11"/>
+      <c r="F17" s="33"/>
+      <c r="G17" s="34"/>
+      <c r="H17" s="33"/>
     </row>
     <row r="18" spans="1:8" ht="31.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5"/>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
       <c r="D18" s="5"/>
-      <c r="E18" s="36" t="s">
+      <c r="E18" s="49" t="s">
         <v>37</v>
       </c>
-      <c r="F18" s="11"/>
-      <c r="G18" s="37"/>
-      <c r="H18" s="11"/>
+      <c r="F18" s="33"/>
+      <c r="G18" s="50"/>
+      <c r="H18" s="33"/>
     </row>
     <row r="19" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="5"/>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
       <c r="D19" s="5"/>
-      <c r="E19" s="17" t="s">
+      <c r="E19" s="52" t="s">
         <v>38</v>
       </c>
-      <c r="F19" s="18"/>
-      <c r="G19" s="49"/>
-      <c r="H19" s="50"/>
+      <c r="F19" s="53"/>
+      <c r="G19" s="56"/>
+      <c r="H19" s="57"/>
     </row>
     <row r="20" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E20" s="19"/>
-      <c r="F20" s="20"/>
-      <c r="G20" s="51"/>
-      <c r="H20" s="52"/>
+      <c r="E20" s="54"/>
+      <c r="F20" s="55"/>
+      <c r="G20" s="58"/>
+      <c r="H20" s="59"/>
     </row>
     <row r="21" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="14" t="s">
+      <c r="A21" s="39" t="s">
         <v>8</v>
       </c>
       <c r="B21" s="9" t="s">
@@ -1247,13 +1159,13 @@
       <c r="E21" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="F21" s="14" t="s">
+      <c r="F21" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="G21" s="55" t="s">
+      <c r="G21" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="H21" s="55"/>
+      <c r="H21" s="13"/>
     </row>
     <row r="22" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="6">
@@ -1263,12 +1175,12 @@
       <c r="C22" s="6"/>
       <c r="D22" s="6"/>
       <c r="E22" s="6"/>
-      <c r="F22" s="48"/>
-      <c r="G22" s="53">
+      <c r="F22" s="10"/>
+      <c r="G22" s="11">
         <f>D22*F22</f>
         <v>0</v>
       </c>
-      <c r="H22" s="54"/>
+      <c r="H22" s="12"/>
     </row>
     <row r="23" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="6">
@@ -1278,12 +1190,12 @@
       <c r="C23" s="6"/>
       <c r="D23" s="6"/>
       <c r="E23" s="6"/>
-      <c r="F23" s="48"/>
-      <c r="G23" s="53">
+      <c r="F23" s="10"/>
+      <c r="G23" s="11">
         <f t="shared" ref="G23:G30" si="0">D23*F23</f>
         <v>0</v>
       </c>
-      <c r="H23" s="54"/>
+      <c r="H23" s="12"/>
     </row>
     <row r="24" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="6">
@@ -1293,12 +1205,12 @@
       <c r="C24" s="6"/>
       <c r="D24" s="6"/>
       <c r="E24" s="6"/>
-      <c r="F24" s="48"/>
-      <c r="G24" s="53">
+      <c r="F24" s="10"/>
+      <c r="G24" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H24" s="54"/>
+      <c r="H24" s="12"/>
     </row>
     <row r="25" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="6">
@@ -1308,12 +1220,12 @@
       <c r="C25" s="6"/>
       <c r="D25" s="6"/>
       <c r="E25" s="6"/>
-      <c r="F25" s="48"/>
-      <c r="G25" s="53">
+      <c r="F25" s="10"/>
+      <c r="G25" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H25" s="54"/>
+      <c r="H25" s="12"/>
     </row>
     <row r="26" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="6">
@@ -1323,12 +1235,12 @@
       <c r="C26" s="6"/>
       <c r="D26" s="6"/>
       <c r="E26" s="6"/>
-      <c r="F26" s="48"/>
-      <c r="G26" s="53">
+      <c r="F26" s="10"/>
+      <c r="G26" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H26" s="54"/>
+      <c r="H26" s="12"/>
     </row>
     <row r="27" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="6">
@@ -1338,12 +1250,12 @@
       <c r="C27" s="6"/>
       <c r="D27" s="6"/>
       <c r="E27" s="6"/>
-      <c r="F27" s="48"/>
-      <c r="G27" s="53">
+      <c r="F27" s="10"/>
+      <c r="G27" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H27" s="54"/>
+      <c r="H27" s="12"/>
     </row>
     <row r="28" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="6">
@@ -1353,12 +1265,12 @@
       <c r="C28" s="6"/>
       <c r="D28" s="6"/>
       <c r="E28" s="6"/>
-      <c r="F28" s="48"/>
-      <c r="G28" s="53">
+      <c r="F28" s="10"/>
+      <c r="G28" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H28" s="54"/>
+      <c r="H28" s="12"/>
     </row>
     <row r="29" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="6">
@@ -1368,12 +1280,12 @@
       <c r="C29" s="6"/>
       <c r="D29" s="6"/>
       <c r="E29" s="6"/>
-      <c r="F29" s="48"/>
-      <c r="G29" s="53">
+      <c r="F29" s="10"/>
+      <c r="G29" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H29" s="54"/>
+      <c r="H29" s="12"/>
     </row>
     <row r="30" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="6">
@@ -1383,12 +1295,12 @@
       <c r="C30" s="6"/>
       <c r="D30" s="6"/>
       <c r="E30" s="6"/>
-      <c r="F30" s="48"/>
-      <c r="G30" s="53">
+      <c r="F30" s="10"/>
+      <c r="G30" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H30" s="54"/>
+      <c r="H30" s="12"/>
     </row>
     <row r="31" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="6">
@@ -1398,12 +1310,12 @@
       <c r="C31" s="6"/>
       <c r="D31" s="6"/>
       <c r="E31" s="6"/>
-      <c r="F31" s="48"/>
-      <c r="G31" s="53">
+      <c r="F31" s="10"/>
+      <c r="G31" s="11">
         <f>D31*F31</f>
         <v>0</v>
       </c>
-      <c r="H31" s="54"/>
+      <c r="H31" s="12"/>
     </row>
     <row r="32" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="6">
@@ -1413,12 +1325,12 @@
       <c r="C32" s="6"/>
       <c r="D32" s="6"/>
       <c r="E32" s="6"/>
-      <c r="F32" s="48"/>
-      <c r="G32" s="53">
+      <c r="F32" s="10"/>
+      <c r="G32" s="11">
         <f>D32*F32</f>
         <v>0</v>
       </c>
-      <c r="H32" s="54"/>
+      <c r="H32" s="12"/>
     </row>
     <row r="33" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="6">
@@ -1428,12 +1340,12 @@
       <c r="C33" s="6"/>
       <c r="D33" s="6"/>
       <c r="E33" s="6"/>
-      <c r="F33" s="48"/>
-      <c r="G33" s="53">
+      <c r="F33" s="10"/>
+      <c r="G33" s="11">
         <f>D33*F33</f>
         <v>0</v>
       </c>
-      <c r="H33" s="54"/>
+      <c r="H33" s="12"/>
     </row>
     <row r="34" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="6">
@@ -1443,271 +1355,271 @@
       <c r="C34" s="6"/>
       <c r="D34" s="6"/>
       <c r="E34" s="6"/>
-      <c r="F34" s="48"/>
-      <c r="G34" s="53">
+      <c r="F34" s="10"/>
+      <c r="G34" s="11">
         <f>D34*F34</f>
         <v>0</v>
       </c>
-      <c r="H34" s="54"/>
+      <c r="H34" s="12"/>
     </row>
     <row r="35" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="36" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="37" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F37" s="34" t="s">
+      <c r="F37" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="G37" s="32"/>
+      <c r="G37" s="19"/>
       <c r="H37" s="1">
         <f>SUM(G22:G34)</f>
         <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F38" s="34" t="s">
+      <c r="F38" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="G38" s="32"/>
+      <c r="G38" s="19"/>
       <c r="H38" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F39" s="34" t="s">
+      <c r="F39" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="G39" s="32"/>
+      <c r="G39" s="19"/>
       <c r="H39" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F40" s="34"/>
-      <c r="G40" s="32"/>
+      <c r="F40" s="25"/>
+      <c r="G40" s="19"/>
       <c r="H40" s="1">
         <f>0.2*(H37+H39)</f>
         <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F41" s="38" t="s">
+      <c r="F41" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="G41" s="32"/>
+      <c r="G41" s="19"/>
       <c r="H41" s="2">
         <f>H37+H39+H40+H38</f>
         <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="41"/>
-      <c r="B42" s="41"/>
-      <c r="C42" s="41"/>
-      <c r="D42" s="41"/>
-      <c r="E42" s="41"/>
-      <c r="F42" s="41"/>
-      <c r="G42" s="41"/>
-      <c r="H42" s="41"/>
+      <c r="A42" s="14"/>
+      <c r="B42" s="14"/>
+      <c r="C42" s="14"/>
+      <c r="D42" s="14"/>
+      <c r="E42" s="14"/>
+      <c r="F42" s="14"/>
+      <c r="G42" s="14"/>
+      <c r="H42" s="14"/>
     </row>
     <row r="43" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="43"/>
-      <c r="B43" s="43"/>
-      <c r="C43" s="43"/>
-      <c r="D43" s="43"/>
-      <c r="E43" s="43"/>
-      <c r="F43" s="43"/>
-      <c r="G43" s="43"/>
-      <c r="H43" s="43"/>
+      <c r="A43" s="16"/>
+      <c r="B43" s="16"/>
+      <c r="C43" s="16"/>
+      <c r="D43" s="16"/>
+      <c r="E43" s="16"/>
+      <c r="F43" s="16"/>
+      <c r="G43" s="16"/>
+      <c r="H43" s="16"/>
     </row>
     <row r="44" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="28" t="s">
+      <c r="A44" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="B44" s="32"/>
-      <c r="C44" s="32"/>
-      <c r="D44" s="32"/>
-      <c r="E44" s="28" t="s">
+      <c r="B44" s="19"/>
+      <c r="C44" s="19"/>
+      <c r="D44" s="19"/>
+      <c r="E44" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="F44" s="32"/>
-      <c r="G44" s="32"/>
-      <c r="H44" s="32"/>
+      <c r="F44" s="19"/>
+      <c r="G44" s="19"/>
+      <c r="H44" s="19"/>
     </row>
     <row r="45" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="33" t="s">
+      <c r="A45" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="B45" s="32"/>
-      <c r="C45" s="32"/>
-      <c r="D45" s="32"/>
-      <c r="E45" s="45" t="s">
+      <c r="B45" s="19"/>
+      <c r="C45" s="19"/>
+      <c r="D45" s="19"/>
+      <c r="E45" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="F45" s="46"/>
-      <c r="G45" s="47"/>
+      <c r="F45" s="22"/>
+      <c r="G45" s="23"/>
       <c r="H45" s="8">
         <f>G18</f>
         <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="33" t="s">
+      <c r="A46" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B46" s="32"/>
-      <c r="C46" s="32"/>
-      <c r="D46" s="32"/>
-      <c r="E46" s="33" t="s">
+      <c r="B46" s="19"/>
+      <c r="C46" s="19"/>
+      <c r="D46" s="19"/>
+      <c r="E46" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="F46" s="32"/>
-      <c r="G46" s="32"/>
-      <c r="H46" s="32"/>
+      <c r="F46" s="19"/>
+      <c r="G46" s="19"/>
+      <c r="H46" s="19"/>
     </row>
     <row r="47" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="33" t="s">
+      <c r="A47" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="B47" s="32"/>
-      <c r="C47" s="32"/>
-      <c r="D47" s="32"/>
-      <c r="E47" s="33" t="s">
+      <c r="B47" s="19"/>
+      <c r="C47" s="19"/>
+      <c r="D47" s="19"/>
+      <c r="E47" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="F47" s="32"/>
-      <c r="G47" s="32"/>
-      <c r="H47" s="32"/>
+      <c r="F47" s="19"/>
+      <c r="G47" s="19"/>
+      <c r="H47" s="19"/>
     </row>
     <row r="48" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="42"/>
-      <c r="B48" s="42"/>
-      <c r="C48" s="42"/>
-      <c r="D48" s="42"/>
-      <c r="E48" s="42"/>
-      <c r="F48" s="42"/>
-      <c r="G48" s="42"/>
-      <c r="H48" s="42"/>
+      <c r="A48" s="15"/>
+      <c r="B48" s="15"/>
+      <c r="C48" s="15"/>
+      <c r="D48" s="15"/>
+      <c r="E48" s="15"/>
+      <c r="F48" s="15"/>
+      <c r="G48" s="15"/>
+      <c r="H48" s="15"/>
     </row>
     <row r="49" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="43"/>
-      <c r="B49" s="43"/>
-      <c r="C49" s="43"/>
-      <c r="D49" s="43"/>
-      <c r="E49" s="43"/>
-      <c r="F49" s="43"/>
-      <c r="G49" s="43"/>
-      <c r="H49" s="43"/>
+      <c r="A49" s="16"/>
+      <c r="B49" s="16"/>
+      <c r="C49" s="16"/>
+      <c r="D49" s="16"/>
+      <c r="E49" s="16"/>
+      <c r="F49" s="16"/>
+      <c r="G49" s="16"/>
+      <c r="H49" s="16"/>
     </row>
     <row r="50" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="28" t="s">
+      <c r="A50" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="B50" s="32"/>
-      <c r="C50" s="32"/>
-      <c r="D50" s="32"/>
-      <c r="E50" s="32"/>
-      <c r="F50" s="32"/>
-      <c r="G50" s="32"/>
-      <c r="H50" s="32"/>
+      <c r="B50" s="19"/>
+      <c r="C50" s="19"/>
+      <c r="D50" s="19"/>
+      <c r="E50" s="19"/>
+      <c r="F50" s="19"/>
+      <c r="G50" s="19"/>
+      <c r="H50" s="19"/>
     </row>
     <row r="51" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="33" t="s">
+      <c r="A51" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="B51" s="32"/>
-      <c r="C51" s="32"/>
-      <c r="D51" s="32"/>
-      <c r="E51" s="32"/>
-      <c r="F51" s="32"/>
-      <c r="G51" s="32"/>
-      <c r="H51" s="32"/>
+      <c r="B51" s="19"/>
+      <c r="C51" s="19"/>
+      <c r="D51" s="19"/>
+      <c r="E51" s="19"/>
+      <c r="F51" s="19"/>
+      <c r="G51" s="19"/>
+      <c r="H51" s="19"/>
     </row>
     <row r="52" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="32"/>
-      <c r="B52" s="32"/>
-      <c r="C52" s="32"/>
-      <c r="D52" s="32"/>
-      <c r="E52" s="32"/>
-      <c r="F52" s="32"/>
-      <c r="G52" s="32"/>
-      <c r="H52" s="32"/>
+      <c r="A52" s="19"/>
+      <c r="B52" s="19"/>
+      <c r="C52" s="19"/>
+      <c r="D52" s="19"/>
+      <c r="E52" s="19"/>
+      <c r="F52" s="19"/>
+      <c r="G52" s="19"/>
+      <c r="H52" s="19"/>
     </row>
     <row r="53" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="32"/>
-      <c r="B53" s="32"/>
-      <c r="C53" s="32"/>
-      <c r="D53" s="32"/>
-      <c r="E53" s="32"/>
-      <c r="F53" s="32"/>
-      <c r="G53" s="32"/>
-      <c r="H53" s="32"/>
+      <c r="A53" s="19"/>
+      <c r="B53" s="19"/>
+      <c r="C53" s="19"/>
+      <c r="D53" s="19"/>
+      <c r="E53" s="19"/>
+      <c r="F53" s="19"/>
+      <c r="G53" s="19"/>
+      <c r="H53" s="19"/>
     </row>
     <row r="54" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="42"/>
-      <c r="B54" s="42"/>
-      <c r="C54" s="42"/>
-      <c r="D54" s="42"/>
-      <c r="E54" s="42"/>
-      <c r="F54" s="42"/>
-      <c r="G54" s="42"/>
-      <c r="H54" s="42"/>
+      <c r="A54" s="15"/>
+      <c r="B54" s="15"/>
+      <c r="C54" s="15"/>
+      <c r="D54" s="15"/>
+      <c r="E54" s="15"/>
+      <c r="F54" s="15"/>
+      <c r="G54" s="15"/>
+      <c r="H54" s="15"/>
     </row>
     <row r="55" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="41"/>
-      <c r="B55" s="41"/>
-      <c r="C55" s="41"/>
-      <c r="D55" s="41"/>
-      <c r="E55" s="41"/>
-      <c r="F55" s="41"/>
-      <c r="G55" s="41"/>
-      <c r="H55" s="41"/>
+      <c r="A55" s="14"/>
+      <c r="B55" s="14"/>
+      <c r="C55" s="14"/>
+      <c r="D55" s="14"/>
+      <c r="E55" s="14"/>
+      <c r="F55" s="14"/>
+      <c r="G55" s="14"/>
+      <c r="H55" s="14"/>
     </row>
     <row r="56" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="44" t="s">
+      <c r="A56" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="B56" s="44"/>
-      <c r="C56" s="44"/>
-      <c r="D56" s="44"/>
-      <c r="E56" s="44" t="s">
+      <c r="B56" s="17"/>
+      <c r="C56" s="17"/>
+      <c r="D56" s="17"/>
+      <c r="E56" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="F56" s="44"/>
-      <c r="G56" s="44"/>
-      <c r="H56" s="44"/>
+      <c r="F56" s="17"/>
+      <c r="G56" s="17"/>
+      <c r="H56" s="17"/>
       <c r="I56" s="3"/>
     </row>
     <row r="57" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="44"/>
-      <c r="B57" s="44"/>
-      <c r="C57" s="44"/>
-      <c r="D57" s="44"/>
-      <c r="E57" s="44"/>
-      <c r="F57" s="44"/>
-      <c r="G57" s="44"/>
-      <c r="H57" s="44"/>
+      <c r="A57" s="17"/>
+      <c r="B57" s="17"/>
+      <c r="C57" s="17"/>
+      <c r="D57" s="17"/>
+      <c r="E57" s="17"/>
+      <c r="F57" s="17"/>
+      <c r="G57" s="17"/>
+      <c r="H57" s="17"/>
       <c r="I57" s="3"/>
     </row>
     <row r="58" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="41"/>
-      <c r="B58" s="41"/>
-      <c r="C58" s="41"/>
-      <c r="D58" s="41"/>
-      <c r="E58" s="41"/>
-      <c r="F58" s="41"/>
-      <c r="G58" s="41"/>
-      <c r="H58" s="41"/>
+      <c r="A58" s="14"/>
+      <c r="B58" s="14"/>
+      <c r="C58" s="14"/>
+      <c r="D58" s="14"/>
+      <c r="E58" s="14"/>
+      <c r="F58" s="14"/>
+      <c r="G58" s="14"/>
+      <c r="H58" s="14"/>
     </row>
     <row r="59" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="30" t="s">
+      <c r="A59" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="B59" s="23"/>
-      <c r="C59" s="23"/>
-      <c r="D59" s="23"/>
-      <c r="E59" s="23"/>
-      <c r="F59" s="23"/>
-      <c r="G59" s="23"/>
-      <c r="H59" s="23"/>
+      <c r="B59" s="36"/>
+      <c r="C59" s="36"/>
+      <c r="D59" s="36"/>
+      <c r="E59" s="36"/>
+      <c r="F59" s="36"/>
+      <c r="G59" s="36"/>
+      <c r="H59" s="36"/>
     </row>
     <row r="60" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="61" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -1750,30 +1662,22 @@
     <row r="98" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="59">
-    <mergeCell ref="A58:H58"/>
-    <mergeCell ref="A48:H49"/>
-    <mergeCell ref="A42:H43"/>
-    <mergeCell ref="E56:H57"/>
-    <mergeCell ref="A56:D57"/>
-    <mergeCell ref="A54:H55"/>
-    <mergeCell ref="A50:H50"/>
-    <mergeCell ref="A45:D45"/>
-    <mergeCell ref="A46:D46"/>
-    <mergeCell ref="E46:H46"/>
-    <mergeCell ref="A44:D44"/>
-    <mergeCell ref="A47:D47"/>
-    <mergeCell ref="E45:G45"/>
-    <mergeCell ref="F41:G41"/>
-    <mergeCell ref="F39:G39"/>
-    <mergeCell ref="F37:G37"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A8:H8"/>
-    <mergeCell ref="C4:H4"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="F7:H7"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="F38:G38"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="C7:E7"/>
+    <mergeCell ref="G9:H10"/>
+    <mergeCell ref="F6:H6"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="C5:H5"/>
+    <mergeCell ref="A9:F10"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="G16:H16"/>
     <mergeCell ref="A59:H59"/>
     <mergeCell ref="A3:B7"/>
     <mergeCell ref="E15:F15"/>
@@ -1788,27 +1692,35 @@
     <mergeCell ref="C3:H3"/>
     <mergeCell ref="C6:E6"/>
     <mergeCell ref="E12:H12"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="C7:E7"/>
-    <mergeCell ref="G9:H10"/>
-    <mergeCell ref="F6:H6"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="C5:H5"/>
     <mergeCell ref="A21"/>
-    <mergeCell ref="A9:F10"/>
-    <mergeCell ref="C14:D14"/>
     <mergeCell ref="E18:F18"/>
+    <mergeCell ref="F41:G41"/>
+    <mergeCell ref="F39:G39"/>
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="C4:H4"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="F7:H7"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="F38:G38"/>
     <mergeCell ref="G18:H18"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="C15:D15"/>
     <mergeCell ref="E19:F20"/>
     <mergeCell ref="G19:H20"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="A58:H58"/>
+    <mergeCell ref="A48:H49"/>
+    <mergeCell ref="A42:H43"/>
+    <mergeCell ref="E56:H57"/>
+    <mergeCell ref="A56:D57"/>
+    <mergeCell ref="A54:H55"/>
+    <mergeCell ref="A50:H50"/>
+    <mergeCell ref="A45:D45"/>
+    <mergeCell ref="A46:D46"/>
+    <mergeCell ref="E46:H46"/>
+    <mergeCell ref="A44:D44"/>
+    <mergeCell ref="A47:D47"/>
+    <mergeCell ref="E45:G45"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.35" bottom="0.35" header="0.2" footer="0.2"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape" r:id="rId1"/>

</xml_diff>